<commit_message>
Se agrega .gitignore y actualización de base de datos a SQLite
</commit_message>
<xml_diff>
--- a/COTIZACION.xlsx
+++ b/COTIZACION.xlsx
@@ -426,90 +426,140 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>PRODUCTO</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>PRECIO</t>
-        </is>
-      </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>PRECIO_BASE</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>PRECIO_VENTA</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>STOCK</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>COMENTARIOS</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>PRODUCTO-1</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="C2" t="n">
+        <v>70</v>
+      </c>
+      <c r="D2" t="n">
         <v>100</v>
       </c>
-      <c r="C2" t="n">
-        <v>1</v>
-      </c>
+      <c r="E2" t="n">
+        <v>20</v>
+      </c>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>PRODUCTO-2</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="C3" t="n">
+        <v>140</v>
+      </c>
+      <c r="D3" t="n">
         <v>200</v>
       </c>
-      <c r="C3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E3" t="n">
+        <v>10</v>
+      </c>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>PRODUCTO-3</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="C4" t="n">
+        <v>210</v>
+      </c>
+      <c r="D4" t="n">
         <v>300</v>
       </c>
-      <c r="C4" t="n">
-        <v>3</v>
-      </c>
+      <c r="E4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>PRODUCTO-4</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="C5" t="n">
+        <v>280</v>
+      </c>
+      <c r="D5" t="n">
         <v>400</v>
       </c>
-      <c r="C5" t="n">
-        <v>4</v>
-      </c>
+      <c r="E5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>PRODUCTO-5</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="C6" t="n">
+        <v>350</v>
+      </c>
+      <c r="D6" t="n">
         <v>500</v>
       </c>
-      <c r="C6" t="n">
-        <v>5</v>
-      </c>
+      <c r="E6" t="n">
+        <v>10</v>
+      </c>
+      <c r="F6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>